<commit_message>
fix: close GT-H3R.1 composite evidence review gap
</commit_message>
<xml_diff>
--- a/docs/golden/gt_h3/remediation/GT_H3R_V5_REVIEW_TABLE.xlsx
+++ b/docs/golden/gt_h3/remediation/GT_H3R_V5_REVIEW_TABLE.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="1" r:id="R2226871b71e04dc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐案复审表" sheetId="2" r:id="R68985083fc4e4ca1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写说明" sheetId="1" r:id="Rfb781eb980c84f5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="逐案复审表" sheetId="2" r:id="Rebb6f860ad714504"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -209,9 +209,9 @@
     <x:tableColumn id="6" name="事件类型"/>
     <x:tableColumn id="7" name="证券代码"/>
     <x:tableColumn id="8" name="交易日"/>
-    <x:tableColumn id="9" name="官方材料名称"/>
-    <x:tableColumn id="10" name="必须核对（按 v5）"/>
-    <x:tableColumn id="11" name="官方链接"/>
+    <x:tableColumn id="9" name="制度规则材料/主官方材料（名称+链接）"/>
+    <x:tableColumn id="10" name="案例适用性材料（复合事实必填，名称+链接）"/>
+    <x:tableColumn id="11" name="必须核对（按 v5）"/>
     <x:tableColumn id="12" name="结果（仅填 APPROVE/REJECT）"/>
     <x:tableColumn id="13" name="简短反馈（REJECT 写原因）"/>
     <x:tableColumn id="14" name="审阅人"/>
@@ -501,31 +501,31 @@
     </x:row>
     <x:row r="12" ht="30" customHeight="1">
       <x:c r="A12" s="11" t="str">
-        <x:v>1. 打开每行官方链接，阅读修正后的官方原文。</x:v>
+        <x:v>1. 打开“制度规则材料/主官方材料”和“案例适用性材料”列中的全部官方原文。</x:v>
       </x:c>
       <x:c r="B12" s="11"/>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="11" t="str">
-        <x:v>2. 对照“必须核对”列检查代码、日期、事件、板块/规则和期望值。</x:v>
+        <x:v>2. AG-025、AG-027、AG-029 的 5 条复合事实必须同时核对规则和案例适用性两份材料。</x:v>
       </x:c>
       <x:c r="B13" s="11"/>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
       <x:c r="A14" s="11" t="str">
-        <x:v>3. 全部一致填 APPROVE；任何不一致填 REJECT 并写一句原因。</x:v>
+        <x:v>3. 对照“必须核对”列检查代码、日期、事件、板块/规则和期望值。</x:v>
       </x:c>
       <x:c r="B14" s="11"/>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
       <x:c r="A15" s="11" t="str">
-        <x:v>4. 12 行完成后填写审阅人和日期，并在 PR 评论明确 12/12 结论。</x:v>
+        <x:v>4. 全部一致填 APPROVE；任何不一致、缺材料或原文不证明事实时填 REJECT 并写一句原因。</x:v>
       </x:c>
       <x:c r="B15" s="11"/>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
       <x:c r="A16" s="11" t="str">
-        <x:v>5. 同时确认 v4 的 113 条 APPROVE 可沿用，以及旧反馈“50”已中和或定义。</x:v>
+        <x:v>5. 12 行完成后填写审阅人和日期，并在 PR 评论明确 12/12 结论、113 条沿用及“50”的处理。</x:v>
       </x:c>
       <x:c r="B16" s="11"/>
     </x:row>
@@ -626,9 +626,9 @@
     <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="13" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="42" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="62" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="52" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="62" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="68" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="60" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="22" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="36" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="16" hidden="0" customWidth="1"/>
@@ -671,13 +671,13 @@
         <x:v>交易日</x:v>
       </x:c>
       <x:c r="I4" s="13" t="str">
-        <x:v>官方材料名称</x:v>
+        <x:v>制度规则材料/主官方材料（名称+链接）</x:v>
       </x:c>
       <x:c r="J4" s="13" t="str">
+        <x:v>案例适用性材料（复合事实必填，名称+链接）</x:v>
+      </x:c>
+      <x:c r="K4" s="13" t="str">
         <x:v>必须核对（按 v5）</x:v>
-      </x:c>
-      <x:c r="K4" s="13" t="str">
-        <x:v>官方链接</x:v>
       </x:c>
       <x:c r="L4" s="13" t="str">
         <x:v>结果（仅填 APPROVE/REJECT）</x:v>
@@ -718,13 +718,15 @@
         <x:v>43619</x:v>
       </x:c>
       <x:c r="I5" s="14" t="str">
-        <x:v>SSE Risk-Warning Board Trading Measures (exact rule page; 5% price-limit clause)</x:v>
+        <x:v>SSE Risk-Warning Board Trading Measures (5% price-limit clause)
+https://www.sse.com.cn/lawandrules/sselawsrules2025/repeal/rules/c/c_20121216_10785153.shtml</x:v>
       </x:c>
       <x:c r="J5" s="14" t="str">
+        <x:v>SSE market disclosure naming 600518 as ST康美 (2019-05-31)
+https://www.sse.com.cn/market/sseindex/diclosure/c/c_20190531_4830732.shtml</x:v>
+      </x:c>
+      <x:c r="K5" s="14" t="str">
         <x:v>核对 600518.SH 在 2019-06-03 是否适用该交易所/板块规则；原文应支持：涨幅上限 5%；跌幅上限 5%。</x:v>
-      </x:c>
-      <x:c r="K5" s="14" t="str">
-        <x:v>https://www.sse.com.cn/lawandrules/sselawsrules2025/repeal/rules/c/c_20121216_10785153.shtml</x:v>
       </x:c>
       <x:c r="L5" s="16" t="str"/>
       <x:c r="M5" s="14" t="str"/>
@@ -757,13 +759,15 @@
         <x:v>43766</x:v>
       </x:c>
       <x:c r="I6" s="14" t="str">
-        <x:v>SSE Risk-Warning Board Trading Measures (exact rule page; 5% price-limit clause)</x:v>
+        <x:v>SSE Risk-Warning Board Trading Measures (5% price-limit clause)
+https://www.sse.com.cn/lawandrules/sselawsrules2025/repeal/rules/c/c_20121216_10785153.shtml</x:v>
       </x:c>
       <x:c r="J6" s="14" t="str">
+        <x:v>SSE 600518 retrospective disclosure (ST status from 2019-05-21)
+https://www.sse.com.cn/disclosure/listedinfo/announcement/c/new/2021-11-27/600518_20211127_2_wfwElR2q.pdf</x:v>
+      </x:c>
+      <x:c r="K6" s="14" t="str">
         <x:v>核对 600518.SH 在 2019-10-28 是否适用该交易所/板块规则；原文应支持：涨幅上限 5%；跌幅上限 5%。</x:v>
-      </x:c>
-      <x:c r="K6" s="14" t="str">
-        <x:v>https://www.sse.com.cn/lawandrules/sselawsrules2025/repeal/rules/c/c_20121216_10785153.shtml</x:v>
       </x:c>
       <x:c r="L6" s="16" t="str"/>
       <x:c r="M6" s="14" t="str"/>
@@ -796,13 +800,14 @@
         <x:v>44348</x:v>
       </x:c>
       <x:c r="I7" s="14" t="str">
-        <x:v>SZSE ChiNext Trading Special Provisions (Notice [2020]515; effective with the 2020-08-24 reform; 20% clause)</x:v>
+        <x:v>SZSE ChiNext Trading Special Provisions (20% clause)
+https://www.szse.cn/lawrules/rule/repeal/rules/P020231230545310237980.pdf</x:v>
       </x:c>
       <x:c r="J7" s="14" t="str">
+        <x:v>—（本行非复合事实）</x:v>
+      </x:c>
+      <x:c r="K7" s="14" t="str">
         <x:v>核对 300750.SZ 在 2021-06-01 是否适用该交易所/板块规则；原文应支持：涨幅上限 20%；跌幅上限 20%。</x:v>
-      </x:c>
-      <x:c r="K7" s="14" t="str">
-        <x:v>https://www.szse.cn/lawrules/rule/repeal/rules/P020231230545310237980.pdf</x:v>
       </x:c>
       <x:c r="L7" s="16" t="str"/>
       <x:c r="M7" s="14" t="str"/>
@@ -835,13 +840,14 @@
         <x:v>44348</x:v>
       </x:c>
       <x:c r="I8" s="14" t="str">
-        <x:v>SZSE ChiNext Trading Special Provisions (Notice [2020]515; effective with the 2020-08-24 reform; 20% clause)</x:v>
+        <x:v>SZSE ChiNext Trading Special Provisions (20% clause)
+https://www.szse.cn/lawrules/rule/repeal/rules/P020231230545310237980.pdf</x:v>
       </x:c>
       <x:c r="J8" s="14" t="str">
+        <x:v>—（本行非复合事实）</x:v>
+      </x:c>
+      <x:c r="K8" s="14" t="str">
         <x:v>核对 300059.SZ 在 2021-06-01 是否适用该交易所/板块规则；原文应支持：涨幅上限 20%；跌幅上限 20%。</x:v>
-      </x:c>
-      <x:c r="K8" s="14" t="str">
-        <x:v>https://www.szse.cn/lawrules/rule/repeal/rules/P020231230545310237980.pdf</x:v>
       </x:c>
       <x:c r="L8" s="16" t="str"/>
       <x:c r="M8" s="14" t="str"/>
@@ -874,13 +880,14 @@
         <x:v>44348</x:v>
       </x:c>
       <x:c r="I9" s="14" t="str">
-        <x:v>SZSE ChiNext Trading Special Provisions (Notice [2020]515; effective with the 2020-08-24 reform; 20% clause)</x:v>
+        <x:v>SZSE ChiNext Trading Special Provisions (20% clause)
+https://www.szse.cn/lawrules/rule/repeal/rules/P020231230545310237980.pdf</x:v>
       </x:c>
       <x:c r="J9" s="14" t="str">
+        <x:v>—（本行非复合事实）</x:v>
+      </x:c>
+      <x:c r="K9" s="14" t="str">
         <x:v>核对 300015.SZ 在 2021-06-01 是否适用该交易所/板块规则；原文应支持：涨幅上限 20%；跌幅上限 20%。</x:v>
-      </x:c>
-      <x:c r="K9" s="14" t="str">
-        <x:v>https://www.szse.cn/lawrules/rule/repeal/rules/P020231230545310237980.pdf</x:v>
       </x:c>
       <x:c r="L9" s="16" t="str"/>
       <x:c r="M9" s="14" t="str"/>
@@ -913,13 +920,14 @@
         <x:v>44348</x:v>
       </x:c>
       <x:c r="I10" s="14" t="str">
-        <x:v>SZSE ChiNext Trading Special Provisions (Notice [2020]515; effective with the 2020-08-24 reform; 20% clause)</x:v>
+        <x:v>SZSE ChiNext Trading Special Provisions (20% clause)
+https://www.szse.cn/lawrules/rule/repeal/rules/P020231230545310237980.pdf</x:v>
       </x:c>
       <x:c r="J10" s="14" t="str">
+        <x:v>—（本行非复合事实）</x:v>
+      </x:c>
+      <x:c r="K10" s="14" t="str">
         <x:v>核对 300124.SZ 在 2021-06-01 是否适用该交易所/板块规则；原文应支持：涨幅上限 20%；跌幅上限 20%。</x:v>
-      </x:c>
-      <x:c r="K10" s="14" t="str">
-        <x:v>https://www.szse.cn/lawrules/rule/repeal/rules/P020231230545310237980.pdf</x:v>
       </x:c>
       <x:c r="L10" s="16" t="str"/>
       <x:c r="M10" s="14" t="str"/>
@@ -952,13 +960,14 @@
         <x:v>44348</x:v>
       </x:c>
       <x:c r="I11" s="14" t="str">
-        <x:v>SZSE ChiNext Trading Special Provisions (Notice [2020]515; effective with the 2020-08-24 reform; 20% clause)</x:v>
+        <x:v>SZSE ChiNext Trading Special Provisions (20% clause)
+https://www.szse.cn/lawrules/rule/repeal/rules/P020231230545310237980.pdf</x:v>
       </x:c>
       <x:c r="J11" s="14" t="str">
+        <x:v>—（本行非复合事实）</x:v>
+      </x:c>
+      <x:c r="K11" s="14" t="str">
         <x:v>核对 300274.SZ 在 2021-06-01 是否适用该交易所/板块规则；原文应支持：涨幅上限 20%；跌幅上限 20%。</x:v>
-      </x:c>
-      <x:c r="K11" s="14" t="str">
-        <x:v>https://www.szse.cn/lawrules/rule/repeal/rules/P020231230545310237980.pdf</x:v>
       </x:c>
       <x:c r="L11" s="16" t="str"/>
       <x:c r="M11" s="14" t="str"/>
@@ -991,13 +1000,15 @@
         <x:v>44035</x:v>
       </x:c>
       <x:c r="I12" s="14" t="str">
-        <x:v>SSE STAR Market Trading Special Provisions (2019; first five listing days no limit, later 20%)</x:v>
+        <x:v>SSE STAR Market Trading Special Provisions (20% after first five days)
+https://www.sse.com.cn/lawandrules/sselawsrules2025/repeal/rules/c/10785118/files/8c544552dc7e4c83a863440179f0b9de.pdf</x:v>
       </x:c>
       <x:c r="J12" s="14" t="str">
+        <x:v>SSE STAR listing notice for 688981 (listed 2020-07-16)
+https://star.sse.com.cn/disclosure/listedinfo/bulletin/star/c/688981_20200715_1.pdf</x:v>
+      </x:c>
+      <x:c r="K12" s="14" t="str">
         <x:v>核对 688981.SH 在 2020-07-23 是否适用该交易所/板块规则；原文应支持：涨幅上限 20%。</x:v>
-      </x:c>
-      <x:c r="K12" s="14" t="str">
-        <x:v>https://www.sse.com.cn/lawandrules/sselawsrules2025/repeal/rules/c/10785118/files/8c544552dc7e4c83a863440179f0b9de.pdf</x:v>
       </x:c>
       <x:c r="L12" s="16" t="str"/>
       <x:c r="M12" s="14" t="str"/>
@@ -1030,13 +1041,15 @@
         <x:v>44137</x:v>
       </x:c>
       <x:c r="I13" s="14" t="str">
-        <x:v>SSE Trading Rules (exact rule page; main-board IPO first-day ±44%/−36% regime)</x:v>
+        <x:v>SSE 2014 new-listing trading supervision notice (44%/36% bounds)
+https://www.sse.com.cn/aboutus/mediacenter/hotandd/c/c_20150912_3988761.shtml</x:v>
       </x:c>
       <x:c r="J13" s="14" t="str">
+        <x:v>SSE official retrospective disclosure for 601995 listing
+https://static.sse.com.cn/disclosure/bond/announcement/company/c/new/2023-04-04/175906_20230404_LS9E.pdf</x:v>
+      </x:c>
+      <x:c r="K13" s="14" t="str">
         <x:v>核对官方原文是否同时证明代码 601995.SH、交易日 2020-11-02 和期望值：涨幅上限 44%；跌幅上限 36%。</x:v>
-      </x:c>
-      <x:c r="K13" s="14" t="str">
-        <x:v>https://www.sse.com.cn/aboutus/mediacenter/hotandd/c/c_20150912_3988761.shtml</x:v>
       </x:c>
       <x:c r="L13" s="16" t="str"/>
       <x:c r="M13" s="14" t="str"/>
@@ -1069,13 +1082,15 @@
         <x:v>44343</x:v>
       </x:c>
       <x:c r="I14" s="14" t="str">
-        <x:v>SSE Trading Rules (exact rule page; main-board IPO first-day ±44%/−36% regime)</x:v>
+        <x:v>SSE 2014 new-listing trading supervision notice (44%/36% bounds)
+https://www.sse.com.cn/aboutus/mediacenter/hotandd/c/c_20150912_3988761.shtml</x:v>
       </x:c>
       <x:c r="J14" s="14" t="str">
+        <x:v>SSE listing announcement for 605499
+https://www.sse.com.cn/disclosure/announcement/listing/ipo/c/c_20210526_81718214.shtml</x:v>
+      </x:c>
+      <x:c r="K14" s="14" t="str">
         <x:v>核对官方原文是否同时证明代码 605499.SH、交易日 2021-05-27 和期望值：涨幅上限 44%；跌幅上限 36%。</x:v>
-      </x:c>
-      <x:c r="K14" s="14" t="str">
-        <x:v>https://www.sse.com.cn/aboutus/mediacenter/hotandd/c/c_20150912_3988761.shtml</x:v>
       </x:c>
       <x:c r="L14" s="16" t="str"/>
       <x:c r="M14" s="14" t="str"/>
@@ -1108,13 +1123,14 @@
         <x:v>44687</x:v>
       </x:c>
       <x:c r="I15" s="14" t="str">
-        <x:v>SZSE official announcement: *ST 科华 risk warning effective 2022-05-06</x:v>
+        <x:v>CNINFO official announcement for 002022 risk warning
+https://static.cninfo.com.cn/finalpage/2022-04-30/1213259774.PDF</x:v>
       </x:c>
       <x:c r="J15" s="14" t="str">
+        <x:v>—（本行非复合事实）</x:v>
+      </x:c>
+      <x:c r="K15" s="14" t="str">
         <x:v>核对官方公告是否明确 002022.SZ 自 2022-05-06 起新增 ST/风险警示；交易日为 2022-05-06，期望值：ST 标记=True。</x:v>
-      </x:c>
-      <x:c r="K15" s="14" t="str">
-        <x:v>https://static.cninfo.com.cn/finalpage/2022-04-30/1213259774.PDF</x:v>
       </x:c>
       <x:c r="L15" s="16" t="str"/>
       <x:c r="M15" s="14" t="str"/>
@@ -1147,13 +1163,14 @@
         <x:v>45408</x:v>
       </x:c>
       <x:c r="I16" s="14" t="str">
-        <x:v>CNINFO official disclosure: *ST 恒宇 risk warning effective 2024-04-26</x:v>
+        <x:v>CNINFO official disclosure for 300965 risk warning
+https://static.cninfo.com.cn/finalpage/2024-04-25/1219804789.PDF</x:v>
       </x:c>
       <x:c r="J16" s="14" t="str">
+        <x:v>—（本行非复合事实）</x:v>
+      </x:c>
+      <x:c r="K16" s="14" t="str">
         <x:v>核对官方公告是否明确 300965.SZ 自 2024-04-26 起新增 ST/风险警示；交易日为 2024-04-26，期望值：ST 标记=True。</x:v>
-      </x:c>
-      <x:c r="K16" s="14" t="str">
-        <x:v>https://static.cninfo.com.cn/finalpage/2024-04-25/1219804789.PDF</x:v>
       </x:c>
       <x:c r="L16" s="16" t="str"/>
       <x:c r="M16" s="14" t="str"/>
@@ -1172,7 +1189,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd015d23285fa417f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rccc2114904614f1f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>